<commit_message>
Auto-deploy AR dashboard 2026-09-14 17:36
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$139</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1352,7 +1352,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Monday, 14 September 2026 - 09:06  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Monday, 14 September 2026 - 17:36  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="9" t="n">
-        <v>125895200651.4888</v>
+        <v>125867357858.2688</v>
       </c>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="10" t="n"/>
@@ -1400,7 +1400,7 @@
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="11" t="n"/>
       <c r="H7" s="13" t="n">
-        <v>10122155929.52296</v>
+        <v>10094313136.30296</v>
       </c>
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="11" t="n"/>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="19" t="n">
-        <v>71428566763.53233</v>
+        <v>71400723970.31233</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="10" t="n"/>
@@ -1517,11 +1517,11 @@
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="27" t="n">
-        <v>9886732972.735821</v>
+        <v>9914575765.95582</v>
       </c>
       <c r="D17" s="11" t="n"/>
       <c r="E17" s="28" t="n">
-        <v>179984164720.4387</v>
+        <v>180243898619.0236</v>
       </c>
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="29" t="n">
@@ -1833,7 +1833,7 @@
         <v>48729455237.06993</v>
       </c>
       <c r="C30" s="35" t="n">
-        <v>8899085906.730999</v>
+        <v>8871243113.511</v>
       </c>
       <c r="D30" s="36" t="n">
         <v>0</v>
@@ -2035,7 +2035,7 @@
         <v>64981293533.39294</v>
       </c>
       <c r="C41" s="50" t="n">
-        <v>6447273230.139372</v>
+        <v>6419430436.919371</v>
       </c>
       <c r="D41" s="51">
         <f>SUM(B41:C41)</f>
@@ -2172,7 +2172,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="58" t="n">
-        <v>8899085906.730999</v>
+        <v>8871243113.511</v>
       </c>
       <c r="J49" s="58">
         <f>SUM(B49:I49)</f>
@@ -3431,7 +3431,7 @@
         <v>5789714193.710999</v>
       </c>
       <c r="D16" s="36" t="n">
-        <v>3109371713.02</v>
+        <v>3081528919.8</v>
       </c>
       <c r="E16" s="36" t="n">
         <v>0</v>
@@ -3476,7 +3476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H139"/>
+  <dimension ref="A1:H138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4941,31 +4941,25 @@
     </row>
     <row r="46">
       <c r="A46" s="73" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="B46" s="74" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C46" s="74" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.SSI/RENTAL/33/2026</t>
-        </is>
-      </c>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C46" s="74" t="n"/>
       <c r="D46" s="74" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E46" s="75" t="n">
-        <v>27842793.22</v>
-      </c>
-      <c r="F46" s="73" t="n">
-        <v>46278</v>
-      </c>
+        <v>13247943944.279</v>
+      </c>
+      <c r="F46" s="73" t="n"/>
       <c r="G46" s="76" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H46" s="74" t="inlineStr">
         <is>
@@ -4989,7 +4983,7 @@
         </is>
       </c>
       <c r="E47" s="75" t="n">
-        <v>13247943944.279</v>
+        <v>1122459338.028</v>
       </c>
       <c r="F47" s="73" t="n"/>
       <c r="G47" s="76" t="n">
@@ -5007,17 +5001,17 @@
       </c>
       <c r="B48" s="74" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C48" s="74" t="n"/>
       <c r="D48" s="74" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E48" s="75" t="n">
-        <v>1122459338.028</v>
+        <v>593353779.5835853</v>
       </c>
       <c r="F48" s="73" t="n"/>
       <c r="G48" s="76" t="n">
@@ -5035,7 +5029,7 @@
       </c>
       <c r="B49" s="74" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C49" s="74" t="n"/>
@@ -5045,7 +5039,7 @@
         </is>
       </c>
       <c r="E49" s="75" t="n">
-        <v>593353779.5835853</v>
+        <v>552691555.2</v>
       </c>
       <c r="F49" s="73" t="n"/>
       <c r="G49" s="76" t="n">
@@ -5101,7 +5095,7 @@
         </is>
       </c>
       <c r="E51" s="75" t="n">
-        <v>552691555.2</v>
+        <v>71167361.40000001</v>
       </c>
       <c r="F51" s="73" t="n"/>
       <c r="G51" s="76" t="n">
@@ -5129,7 +5123,7 @@
         </is>
       </c>
       <c r="E52" s="75" t="n">
-        <v>71167361.40000001</v>
+        <v>299652048</v>
       </c>
       <c r="F52" s="73" t="n"/>
       <c r="G52" s="76" t="n">
@@ -5153,11 +5147,11 @@
       <c r="C53" s="74" t="n"/>
       <c r="D53" s="74" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E53" s="75" t="n">
-        <v>299652048</v>
+        <v>5789714193.710999</v>
       </c>
       <c r="F53" s="73" t="n"/>
       <c r="G53" s="76" t="n">
@@ -5181,11 +5175,11 @@
       <c r="C54" s="74" t="n"/>
       <c r="D54" s="74" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E54" s="75" t="n">
-        <v>5789714193.710999</v>
+        <v>1605326400</v>
       </c>
       <c r="F54" s="73" t="n"/>
       <c r="G54" s="76" t="n">
@@ -5198,30 +5192,36 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="73" t="n">
-        <v>46279</v>
-      </c>
-      <c r="B55" s="74" t="inlineStr">
+      <c r="A55" s="77" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B55" s="78" t="inlineStr">
         <is>
           <t>PT Syngenta Indonesia</t>
         </is>
       </c>
-      <c r="C55" s="74" t="n"/>
-      <c r="D55" s="74" t="inlineStr">
-        <is>
-          <t>Rental</t>
-        </is>
-      </c>
-      <c r="E55" s="75" t="n">
-        <v>1605326400</v>
-      </c>
-      <c r="F55" s="73" t="n"/>
-      <c r="G55" s="76" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="74" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="C55" s="78" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
+        </is>
+      </c>
+      <c r="D55" s="78" t="inlineStr">
+        <is>
+          <t>Tolling</t>
+        </is>
+      </c>
+      <c r="E55" s="79" t="n">
+        <v>326395903.6008</v>
+      </c>
+      <c r="F55" s="77" t="n">
+        <v>46284</v>
+      </c>
+      <c r="G55" s="80" t="n">
+        <v>5</v>
+      </c>
+      <c r="H55" s="78" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="C56" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
         </is>
       </c>
       <c r="D56" s="78" t="inlineStr">
@@ -5245,7 +5245,7 @@
         </is>
       </c>
       <c r="E56" s="79" t="n">
-        <v>326395903.6008</v>
+        <v>240049.20888</v>
       </c>
       <c r="F56" s="77" t="n">
         <v>46284</v>
@@ -5261,7 +5261,7 @@
     </row>
     <row r="57">
       <c r="A57" s="77" t="n">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="B57" s="78" t="inlineStr">
         <is>
@@ -5270,7 +5270,7 @@
       </c>
       <c r="C57" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
         </is>
       </c>
       <c r="D57" s="78" t="inlineStr">
@@ -5279,13 +5279,13 @@
         </is>
       </c>
       <c r="E57" s="79" t="n">
-        <v>240049.20888</v>
+        <v>570800977.7184</v>
       </c>
       <c r="F57" s="77" t="n">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="G57" s="80" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H57" s="78" t="inlineStr">
         <is>
@@ -5295,16 +5295,16 @@
     </row>
     <row r="58">
       <c r="A58" s="77" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="B58" s="78" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C58" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
+          <t>PT.PSI/PT.CASI/REP/53/2026</t>
         </is>
       </c>
       <c r="D58" s="78" t="inlineStr">
@@ -5313,13 +5313,13 @@
         </is>
       </c>
       <c r="E58" s="79" t="n">
-        <v>570800977.7184</v>
+        <v>36849832.74</v>
       </c>
       <c r="F58" s="77" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="G58" s="80" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H58" s="78" t="inlineStr">
         <is>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="C59" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/53/2026</t>
+          <t>PT.PSI/PT.CASI/REP/54/2026</t>
         </is>
       </c>
       <c r="D59" s="78" t="inlineStr">
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="E59" s="79" t="n">
-        <v>36849832.74</v>
+        <v>31988016.36</v>
       </c>
       <c r="F59" s="77" t="n">
         <v>46285</v>
@@ -5372,7 +5372,7 @@
       </c>
       <c r="C60" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/54/2026</t>
+          <t>PT.PSI/PT.CASI/REP/55/2026</t>
         </is>
       </c>
       <c r="D60" s="78" t="inlineStr">
@@ -5381,7 +5381,7 @@
         </is>
       </c>
       <c r="E60" s="79" t="n">
-        <v>31988016.36</v>
+        <v>19431065.722</v>
       </c>
       <c r="F60" s="77" t="n">
         <v>46285</v>
@@ -5397,16 +5397,16 @@
     </row>
     <row r="61">
       <c r="A61" s="77" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B61" s="78" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C61" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/55/2026</t>
+          <t>PT.PSI/PT.BI/FC/43/2026</t>
         </is>
       </c>
       <c r="D61" s="78" t="inlineStr">
@@ -5415,13 +5415,13 @@
         </is>
       </c>
       <c r="E61" s="79" t="n">
-        <v>19431065.722</v>
+        <v>103679056</v>
       </c>
       <c r="F61" s="77" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="G61" s="80" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H61" s="78" t="inlineStr">
         <is>
@@ -5440,7 +5440,7 @@
       </c>
       <c r="C62" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/43/2026</t>
+          <t>PT.PSI/PT.BI/FC/44/2026</t>
         </is>
       </c>
       <c r="D62" s="78" t="inlineStr">
@@ -5449,7 +5449,7 @@
         </is>
       </c>
       <c r="E62" s="79" t="n">
-        <v>103679056</v>
+        <v>92863095</v>
       </c>
       <c r="F62" s="77" t="n">
         <v>46292</v>
@@ -5474,7 +5474,7 @@
       </c>
       <c r="C63" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/44/2026</t>
+          <t>PT.PSI/PT.BI/FC/45/2026</t>
         </is>
       </c>
       <c r="D63" s="78" t="inlineStr">
@@ -5483,7 +5483,7 @@
         </is>
       </c>
       <c r="E63" s="79" t="n">
-        <v>92863095</v>
+        <v>17392258</v>
       </c>
       <c r="F63" s="77" t="n">
         <v>46292</v>
@@ -5508,7 +5508,7 @@
       </c>
       <c r="C64" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/45/2026</t>
+          <t>PT.PSI/PT.BI/FC/46/2026</t>
         </is>
       </c>
       <c r="D64" s="78" t="inlineStr">
@@ -5517,7 +5517,7 @@
         </is>
       </c>
       <c r="E64" s="79" t="n">
-        <v>17392258</v>
+        <v>197734556.5</v>
       </c>
       <c r="F64" s="77" t="n">
         <v>46292</v>
@@ -5542,7 +5542,7 @@
       </c>
       <c r="C65" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/46/2026</t>
+          <t>PT.PSI/PT.BI/FC/47/2026</t>
         </is>
       </c>
       <c r="D65" s="78" t="inlineStr">
@@ -5551,7 +5551,7 @@
         </is>
       </c>
       <c r="E65" s="79" t="n">
-        <v>197734556.5</v>
+        <v>254755628.4</v>
       </c>
       <c r="F65" s="77" t="n">
         <v>46292</v>
@@ -5576,7 +5576,7 @@
       </c>
       <c r="C66" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/47/2026</t>
+          <t>PT.PSI/PT.BI/FC/48/2026</t>
         </is>
       </c>
       <c r="D66" s="78" t="inlineStr">
@@ -5585,7 +5585,7 @@
         </is>
       </c>
       <c r="E66" s="79" t="n">
-        <v>254755628.4</v>
+        <v>10599160</v>
       </c>
       <c r="F66" s="77" t="n">
         <v>46292</v>
@@ -5610,7 +5610,7 @@
       </c>
       <c r="C67" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/48/2026</t>
+          <t>PT.PSI/PT.BI/FC/49/2026</t>
         </is>
       </c>
       <c r="D67" s="78" t="inlineStr">
@@ -5619,7 +5619,7 @@
         </is>
       </c>
       <c r="E67" s="79" t="n">
-        <v>10599160</v>
+        <v>54405006.5</v>
       </c>
       <c r="F67" s="77" t="n">
         <v>46292</v>
@@ -5644,7 +5644,7 @@
       </c>
       <c r="C68" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/49/2026</t>
+          <t>PT.PSI/PT.BI/FC/50/2026</t>
         </is>
       </c>
       <c r="D68" s="78" t="inlineStr">
@@ -5653,7 +5653,7 @@
         </is>
       </c>
       <c r="E68" s="79" t="n">
-        <v>54405006.5</v>
+        <v>1075481.2</v>
       </c>
       <c r="F68" s="77" t="n">
         <v>46292</v>
@@ -5678,7 +5678,7 @@
       </c>
       <c r="C69" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/50/2026</t>
+          <t>PT.PSI/PT.BI/FC/51/2026</t>
         </is>
       </c>
       <c r="D69" s="78" t="inlineStr">
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="E69" s="79" t="n">
-        <v>1075481.2</v>
+        <v>803447.72</v>
       </c>
       <c r="F69" s="77" t="n">
         <v>46292</v>
@@ -5712,7 +5712,7 @@
       </c>
       <c r="C70" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/51/2026</t>
+          <t>PT.PSI/PT.BI/FC/52/2026</t>
         </is>
       </c>
       <c r="D70" s="78" t="inlineStr">
@@ -5721,7 +5721,7 @@
         </is>
       </c>
       <c r="E70" s="79" t="n">
-        <v>803447.72</v>
+        <v>7250789</v>
       </c>
       <c r="F70" s="77" t="n">
         <v>46292</v>
@@ -5746,7 +5746,7 @@
       </c>
       <c r="C71" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/52/2026</t>
+          <t>PT.PSI/PT.BI/FC/53/2026</t>
         </is>
       </c>
       <c r="D71" s="78" t="inlineStr">
@@ -5755,7 +5755,7 @@
         </is>
       </c>
       <c r="E71" s="79" t="n">
-        <v>7250789</v>
+        <v>101318334</v>
       </c>
       <c r="F71" s="77" t="n">
         <v>46292</v>
@@ -5771,7 +5771,7 @@
     </row>
     <row r="72">
       <c r="A72" s="77" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B72" s="78" t="inlineStr">
         <is>
@@ -5780,7 +5780,7 @@
       </c>
       <c r="C72" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/53/2026</t>
+          <t>PT.PSI/PT.BI/FC/54/2026</t>
         </is>
       </c>
       <c r="D72" s="78" t="inlineStr">
@@ -5789,13 +5789,13 @@
         </is>
       </c>
       <c r="E72" s="79" t="n">
-        <v>101318334</v>
+        <v>156400274.1</v>
       </c>
       <c r="F72" s="77" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G72" s="80" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H72" s="78" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C73" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/54/2026</t>
+          <t>PT.PSI/PT.BI/FC/55/2026</t>
         </is>
       </c>
       <c r="D73" s="78" t="inlineStr">
@@ -5823,7 +5823,7 @@
         </is>
       </c>
       <c r="E73" s="79" t="n">
-        <v>156400274.1</v>
+        <v>50838199.5</v>
       </c>
       <c r="F73" s="77" t="n">
         <v>46293</v>
@@ -5848,7 +5848,7 @@
       </c>
       <c r="C74" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/55/2026</t>
+          <t>PT.PSI/PT.BI/FC/56/2026</t>
         </is>
       </c>
       <c r="D74" s="78" t="inlineStr">
@@ -5857,7 +5857,7 @@
         </is>
       </c>
       <c r="E74" s="79" t="n">
-        <v>50838199.5</v>
+        <v>376884765.6</v>
       </c>
       <c r="F74" s="77" t="n">
         <v>46293</v>
@@ -5882,7 +5882,7 @@
       </c>
       <c r="C75" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/56/2026</t>
+          <t>PT.PSI/PT.BI/FC/57/2026</t>
         </is>
       </c>
       <c r="D75" s="78" t="inlineStr">
@@ -5891,7 +5891,7 @@
         </is>
       </c>
       <c r="E75" s="79" t="n">
-        <v>376884765.6</v>
+        <v>100336789</v>
       </c>
       <c r="F75" s="77" t="n">
         <v>46293</v>
@@ -5916,7 +5916,7 @@
       </c>
       <c r="C76" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/57/2026</t>
+          <t>PT.PSI/PT.BI/FC/58/2026</t>
         </is>
       </c>
       <c r="D76" s="78" t="inlineStr">
@@ -5925,7 +5925,7 @@
         </is>
       </c>
       <c r="E76" s="79" t="n">
-        <v>100336789</v>
+        <v>787756603.1999999</v>
       </c>
       <c r="F76" s="77" t="n">
         <v>46293</v>
@@ -5950,7 +5950,7 @@
       </c>
       <c r="C77" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/58/2026</t>
+          <t>PT.PSI/PT.BI/FC/59/2026</t>
         </is>
       </c>
       <c r="D77" s="78" t="inlineStr">
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="E77" s="79" t="n">
-        <v>787756603.1999999</v>
+        <v>140859991.5</v>
       </c>
       <c r="F77" s="77" t="n">
         <v>46293</v>
@@ -5975,16 +5975,16 @@
     </row>
     <row r="78">
       <c r="A78" s="77" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="B78" s="78" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C78" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/59/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/66/2026 </t>
         </is>
       </c>
       <c r="D78" s="78" t="inlineStr">
@@ -5993,13 +5993,13 @@
         </is>
       </c>
       <c r="E78" s="79" t="n">
-        <v>140859991.5</v>
+        <v>3100200501.96</v>
       </c>
       <c r="F78" s="77" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="G78" s="80" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H78" s="78" t="inlineStr">
         <is>
@@ -6018,7 +6018,7 @@
       </c>
       <c r="C79" s="78" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/66/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
         </is>
       </c>
       <c r="D79" s="78" t="inlineStr">
@@ -6027,7 +6027,7 @@
         </is>
       </c>
       <c r="E79" s="79" t="n">
-        <v>3100200501.96</v>
+        <v>237729</v>
       </c>
       <c r="F79" s="77" t="n">
         <v>46296</v>
@@ -6061,7 +6061,7 @@
         </is>
       </c>
       <c r="E80" s="79" t="n">
-        <v>237729</v>
+        <v>142404425.58</v>
       </c>
       <c r="F80" s="77" t="n">
         <v>46296</v>
@@ -6095,7 +6095,7 @@
         </is>
       </c>
       <c r="E81" s="79" t="n">
-        <v>142404425.58</v>
+        <v>270535602</v>
       </c>
       <c r="F81" s="77" t="n">
         <v>46296</v>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="C82" s="78" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/68/2026 </t>
         </is>
       </c>
       <c r="D82" s="78" t="inlineStr">
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="E82" s="79" t="n">
-        <v>270535602</v>
+        <v>28798491.06</v>
       </c>
       <c r="F82" s="77" t="n">
         <v>46296</v>
@@ -6149,24 +6149,24 @@
       </c>
       <c r="B83" s="78" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C83" s="78" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/68/2026 </t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/13/2026</t>
         </is>
       </c>
       <c r="D83" s="78" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E83" s="79" t="n">
-        <v>28798491.06</v>
+        <v>872911811.2</v>
       </c>
       <c r="F83" s="77" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="G83" s="80" t="n">
         <v>17</v>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="C84" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/13/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/14/2026</t>
         </is>
       </c>
       <c r="D84" s="78" t="inlineStr">
@@ -6197,7 +6197,7 @@
         </is>
       </c>
       <c r="E84" s="79" t="n">
-        <v>872911811.2</v>
+        <v>302161780.8</v>
       </c>
       <c r="F84" s="77" t="n">
         <v>46295</v>
@@ -6213,16 +6213,16 @@
     </row>
     <row r="85">
       <c r="A85" s="77" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="B85" s="78" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C85" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/14/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
         </is>
       </c>
       <c r="D85" s="78" t="inlineStr">
@@ -6231,13 +6231,13 @@
         </is>
       </c>
       <c r="E85" s="79" t="n">
-        <v>302161780.8</v>
+        <v>18871809.6</v>
       </c>
       <c r="F85" s="77" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="G85" s="80" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H85" s="78" t="inlineStr">
         <is>
@@ -6247,7 +6247,7 @@
     </row>
     <row r="86">
       <c r="A86" s="77" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B86" s="78" t="inlineStr">
         <is>
@@ -6256,22 +6256,22 @@
       </c>
       <c r="C86" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
         </is>
       </c>
       <c r="D86" s="78" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E86" s="79" t="n">
-        <v>18871809.6</v>
+        <v>226017285.066</v>
       </c>
       <c r="F86" s="77" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="G86" s="80" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H86" s="78" t="inlineStr">
         <is>
@@ -6290,7 +6290,7 @@
       </c>
       <c r="C87" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
         </is>
       </c>
       <c r="D87" s="78" t="inlineStr">
@@ -6299,7 +6299,7 @@
         </is>
       </c>
       <c r="E87" s="79" t="n">
-        <v>226017285.066</v>
+        <v>3356193038.598001</v>
       </c>
       <c r="F87" s="77" t="n">
         <v>46301</v>
@@ -6324,7 +6324,7 @@
       </c>
       <c r="C88" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
         </is>
       </c>
       <c r="D88" s="78" t="inlineStr">
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="E88" s="79" t="n">
-        <v>3356193038.598001</v>
+        <v>767489805.3095999</v>
       </c>
       <c r="F88" s="77" t="n">
         <v>46301</v>
@@ -6367,7 +6367,7 @@
         </is>
       </c>
       <c r="E89" s="79" t="n">
-        <v>767489805.3095999</v>
+        <v>231565952.52</v>
       </c>
       <c r="F89" s="77" t="n">
         <v>46301</v>
@@ -6383,31 +6383,31 @@
     </row>
     <row r="90">
       <c r="A90" s="77" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="B90" s="78" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C90" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/15/2026</t>
         </is>
       </c>
       <c r="D90" s="78" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E90" s="79" t="n">
-        <v>231565952.52</v>
+        <v>541504029.249372</v>
       </c>
       <c r="F90" s="77" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G90" s="80" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H90" s="78" t="inlineStr">
         <is>
@@ -6426,7 +6426,7 @@
       </c>
       <c r="C91" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/15/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL OFFICE/03/2026</t>
         </is>
       </c>
       <c r="D91" s="78" t="inlineStr">
@@ -6435,7 +6435,7 @@
         </is>
       </c>
       <c r="E91" s="79" t="n">
-        <v>541504029.249372</v>
+        <v>22509333.69</v>
       </c>
       <c r="F91" s="77" t="n">
         <v>46298</v>
@@ -6451,16 +6451,16 @@
     </row>
     <row r="92">
       <c r="A92" s="77" t="n">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="B92" s="78" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C92" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL OFFICE/03/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-25/IX/2026</t>
         </is>
       </c>
       <c r="D92" s="78" t="inlineStr">
@@ -6469,13 +6469,13 @@
         </is>
       </c>
       <c r="E92" s="79" t="n">
-        <v>22509333.69</v>
+        <v>816231500</v>
       </c>
       <c r="F92" s="77" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="G92" s="80" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H92" s="78" t="inlineStr">
         <is>
@@ -6494,7 +6494,7 @@
       </c>
       <c r="C93" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-25/IX/2026</t>
+          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
         </is>
       </c>
       <c r="D93" s="78" t="inlineStr">
@@ -6503,7 +6503,7 @@
         </is>
       </c>
       <c r="E93" s="79" t="n">
-        <v>816231500</v>
+        <v>11590259.94</v>
       </c>
       <c r="F93" s="77" t="n">
         <v>46305</v>
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="E94" s="79" t="n">
-        <v>11590259.94</v>
+        <v>62675</v>
       </c>
       <c r="F94" s="77" t="n">
         <v>46305</v>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="C95" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/27/IX/2026</t>
         </is>
       </c>
       <c r="D95" s="78" t="inlineStr">
@@ -6571,7 +6571,7 @@
         </is>
       </c>
       <c r="E95" s="79" t="n">
-        <v>62675</v>
+        <v>755480000</v>
       </c>
       <c r="F95" s="77" t="n">
         <v>46305</v>
@@ -6591,21 +6591,21 @@
       </c>
       <c r="B96" s="78" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C96" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/27/IX/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/12/2026</t>
         </is>
       </c>
       <c r="D96" s="78" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E96" s="79" t="n">
-        <v>755480000</v>
+        <v>802240</v>
       </c>
       <c r="F96" s="77" t="n">
         <v>46305</v>
@@ -6630,7 +6630,7 @@
       </c>
       <c r="C97" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/12/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/13/2026</t>
         </is>
       </c>
       <c r="D97" s="78" t="inlineStr">
@@ -6639,7 +6639,7 @@
         </is>
       </c>
       <c r="E97" s="79" t="n">
-        <v>802240</v>
+        <v>8632800</v>
       </c>
       <c r="F97" s="77" t="n">
         <v>46305</v>
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C98" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/13/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/14/2026</t>
         </is>
       </c>
       <c r="D98" s="78" t="inlineStr">
@@ -6673,7 +6673,7 @@
         </is>
       </c>
       <c r="E98" s="79" t="n">
-        <v>8632800</v>
+        <v>967920</v>
       </c>
       <c r="F98" s="77" t="n">
         <v>46305</v>
@@ -6698,7 +6698,7 @@
       </c>
       <c r="C99" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/14/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/15/2026</t>
         </is>
       </c>
       <c r="D99" s="78" t="inlineStr">
@@ -6707,7 +6707,7 @@
         </is>
       </c>
       <c r="E99" s="79" t="n">
-        <v>967920</v>
+        <v>20509440</v>
       </c>
       <c r="F99" s="77" t="n">
         <v>46305</v>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="C100" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/15/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/16/2026</t>
         </is>
       </c>
       <c r="D100" s="78" t="inlineStr">
@@ -6741,7 +6741,7 @@
         </is>
       </c>
       <c r="E100" s="79" t="n">
-        <v>20509440</v>
+        <v>2180000</v>
       </c>
       <c r="F100" s="77" t="n">
         <v>46305</v>
@@ -6766,7 +6766,7 @@
       </c>
       <c r="C101" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/16/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/17/2026</t>
         </is>
       </c>
       <c r="D101" s="78" t="inlineStr">
@@ -6775,7 +6775,7 @@
         </is>
       </c>
       <c r="E101" s="79" t="n">
-        <v>2180000</v>
+        <v>540640</v>
       </c>
       <c r="F101" s="77" t="n">
         <v>46305</v>
@@ -6800,7 +6800,7 @@
       </c>
       <c r="C102" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/17/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/18/2026</t>
         </is>
       </c>
       <c r="D102" s="78" t="inlineStr">
@@ -6809,7 +6809,7 @@
         </is>
       </c>
       <c r="E102" s="79" t="n">
-        <v>540640</v>
+        <v>47532720</v>
       </c>
       <c r="F102" s="77" t="n">
         <v>46305</v>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="C103" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/18/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/19/2026</t>
         </is>
       </c>
       <c r="D103" s="78" t="inlineStr">
@@ -6843,7 +6843,7 @@
         </is>
       </c>
       <c r="E103" s="79" t="n">
-        <v>47532720</v>
+        <v>50794000</v>
       </c>
       <c r="F103" s="77" t="n">
         <v>46305</v>
@@ -6863,12 +6863,12 @@
       </c>
       <c r="B104" s="78" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C104" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/19/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
         </is>
       </c>
       <c r="D104" s="78" t="inlineStr">
@@ -6877,7 +6877,7 @@
         </is>
       </c>
       <c r="E104" s="79" t="n">
-        <v>50794000</v>
+        <v>886307502.1920002</v>
       </c>
       <c r="F104" s="77" t="n">
         <v>46305</v>
@@ -6893,7 +6893,7 @@
     </row>
     <row r="105">
       <c r="A105" s="77" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B105" s="78" t="inlineStr">
         <is>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="C105" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
         </is>
       </c>
       <c r="D105" s="78" t="inlineStr">
@@ -6911,13 +6911,13 @@
         </is>
       </c>
       <c r="E105" s="79" t="n">
-        <v>886307502.1920002</v>
+        <v>5676698527.872001</v>
       </c>
       <c r="F105" s="77" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="G105" s="80" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="H105" s="78" t="inlineStr">
         <is>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="C106" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
         </is>
       </c>
       <c r="D106" s="78" t="inlineStr">
@@ -6945,7 +6945,7 @@
         </is>
       </c>
       <c r="E106" s="79" t="n">
-        <v>5676698527.872001</v>
+        <v>564189103.6416</v>
       </c>
       <c r="F106" s="77" t="n">
         <v>46308</v>
@@ -6961,16 +6961,16 @@
     </row>
     <row r="107">
       <c r="A107" s="77" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="B107" s="78" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C107" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
+          <t>PT.PSI/PT.CASI/REP/56/2026</t>
         </is>
       </c>
       <c r="D107" s="78" t="inlineStr">
@@ -6979,13 +6979,13 @@
         </is>
       </c>
       <c r="E107" s="79" t="n">
-        <v>564189103.6416</v>
+        <v>5535207.48</v>
       </c>
       <c r="F107" s="77" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="G107" s="80" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H107" s="78" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
       </c>
       <c r="C108" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/56/2026</t>
+          <t>PT.PSI/PT.CASI/REP/57/2026</t>
         </is>
       </c>
       <c r="D108" s="78" t="inlineStr">
@@ -7013,7 +7013,7 @@
         </is>
       </c>
       <c r="E108" s="79" t="n">
-        <v>5535207.48</v>
+        <v>4392388.26</v>
       </c>
       <c r="F108" s="77" t="n">
         <v>46304</v>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="C109" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/57/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/58/2026</t>
         </is>
       </c>
       <c r="D109" s="78" t="inlineStr">
@@ -7047,7 +7047,7 @@
         </is>
       </c>
       <c r="E109" s="79" t="n">
-        <v>4392388.26</v>
+        <v>18129124.98186</v>
       </c>
       <c r="F109" s="77" t="n">
         <v>46304</v>
@@ -7072,7 +7072,7 @@
       </c>
       <c r="C110" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/58/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/59/2026</t>
         </is>
       </c>
       <c r="D110" s="78" t="inlineStr">
@@ -7081,7 +7081,7 @@
         </is>
       </c>
       <c r="E110" s="79" t="n">
-        <v>18129124.98186</v>
+        <v>9884824431.36027</v>
       </c>
       <c r="F110" s="77" t="n">
         <v>46304</v>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="C111" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/59/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/60/2026</t>
         </is>
       </c>
       <c r="D111" s="78" t="inlineStr">
@@ -7115,7 +7115,7 @@
         </is>
       </c>
       <c r="E111" s="79" t="n">
-        <v>9884824431.36027</v>
+        <v>700304033.0543</v>
       </c>
       <c r="F111" s="77" t="n">
         <v>46304</v>
@@ -7140,7 +7140,7 @@
       </c>
       <c r="C112" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/60/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/61/2026</t>
         </is>
       </c>
       <c r="D112" s="78" t="inlineStr">
@@ -7149,7 +7149,7 @@
         </is>
       </c>
       <c r="E112" s="79" t="n">
-        <v>700304033.0543</v>
+        <v>1147400616.7888</v>
       </c>
       <c r="F112" s="77" t="n">
         <v>46304</v>
@@ -7174,7 +7174,7 @@
       </c>
       <c r="C113" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/61/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/62/2026</t>
         </is>
       </c>
       <c r="D113" s="78" t="inlineStr">
@@ -7183,7 +7183,7 @@
         </is>
       </c>
       <c r="E113" s="79" t="n">
-        <v>1147400616.7888</v>
+        <v>4999029.5912</v>
       </c>
       <c r="F113" s="77" t="n">
         <v>46304</v>
@@ -7208,7 +7208,7 @@
       </c>
       <c r="C114" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/62/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/63/2026</t>
         </is>
       </c>
       <c r="D114" s="78" t="inlineStr">
@@ -7217,7 +7217,7 @@
         </is>
       </c>
       <c r="E114" s="79" t="n">
-        <v>4999029.5912</v>
+        <v>34933281.3146</v>
       </c>
       <c r="F114" s="77" t="n">
         <v>46304</v>
@@ -7242,7 +7242,7 @@
       </c>
       <c r="C115" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/63/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/64/2026</t>
         </is>
       </c>
       <c r="D115" s="78" t="inlineStr">
@@ -7251,7 +7251,7 @@
         </is>
       </c>
       <c r="E115" s="79" t="n">
-        <v>34933281.3146</v>
+        <v>85105002.66900001</v>
       </c>
       <c r="F115" s="77" t="n">
         <v>46304</v>
@@ -7276,7 +7276,7 @@
       </c>
       <c r="C116" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/64/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/65/2026</t>
         </is>
       </c>
       <c r="D116" s="78" t="inlineStr">
@@ -7285,7 +7285,7 @@
         </is>
       </c>
       <c r="E116" s="79" t="n">
-        <v>85105002.66900001</v>
+        <v>886098780.5445001</v>
       </c>
       <c r="F116" s="77" t="n">
         <v>46304</v>
@@ -7310,7 +7310,7 @@
       </c>
       <c r="C117" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/65/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/66/2026</t>
         </is>
       </c>
       <c r="D117" s="78" t="inlineStr">
@@ -7319,7 +7319,7 @@
         </is>
       </c>
       <c r="E117" s="79" t="n">
-        <v>886098780.5445001</v>
+        <v>262631.43648</v>
       </c>
       <c r="F117" s="77" t="n">
         <v>46304</v>
@@ -7335,31 +7335,31 @@
     </row>
     <row r="118">
       <c r="A118" s="77" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="B118" s="78" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C118" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/66/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
         </is>
       </c>
       <c r="D118" s="78" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E118" s="79" t="n">
-        <v>262631.43648</v>
+        <v>1365520000</v>
       </c>
       <c r="F118" s="77" t="n">
-        <v>46304</v>
+        <v>46312</v>
       </c>
       <c r="G118" s="80" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H118" s="78" t="inlineStr">
         <is>
@@ -7378,7 +7378,7 @@
       </c>
       <c r="C119" s="78" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
         </is>
       </c>
       <c r="D119" s="78" t="inlineStr">
@@ -7387,7 +7387,7 @@
         </is>
       </c>
       <c r="E119" s="79" t="n">
-        <v>1365520000</v>
+        <v>9687031.199999999</v>
       </c>
       <c r="F119" s="77" t="n">
         <v>46312</v>
@@ -7412,7 +7412,7 @@
       </c>
       <c r="C120" s="78" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
         </is>
       </c>
       <c r="D120" s="78" t="inlineStr">
@@ -7421,7 +7421,7 @@
         </is>
       </c>
       <c r="E120" s="79" t="n">
-        <v>9687031.199999999</v>
+        <v>1070726250</v>
       </c>
       <c r="F120" s="77" t="n">
         <v>46312</v>
@@ -7446,7 +7446,7 @@
       </c>
       <c r="C121" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
         </is>
       </c>
       <c r="D121" s="78" t="inlineStr">
@@ -7455,7 +7455,7 @@
         </is>
       </c>
       <c r="E121" s="79" t="n">
-        <v>1070726250</v>
+        <v>272700000</v>
       </c>
       <c r="F121" s="77" t="n">
         <v>46312</v>
@@ -7471,7 +7471,7 @@
     </row>
     <row r="122">
       <c r="A122" s="77" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B122" s="78" t="inlineStr">
         <is>
@@ -7480,22 +7480,22 @@
       </c>
       <c r="C122" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
         </is>
       </c>
       <c r="D122" s="78" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E122" s="79" t="n">
-        <v>272700000</v>
+        <v>545818781.4912</v>
       </c>
       <c r="F122" s="77" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="G122" s="80" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H122" s="78" t="inlineStr">
         <is>
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C123" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
         </is>
       </c>
       <c r="D123" s="78" t="inlineStr">
@@ -7523,7 +7523,7 @@
         </is>
       </c>
       <c r="E123" s="79" t="n">
-        <v>545818781.4912</v>
+        <v>767367847.5204</v>
       </c>
       <c r="F123" s="77" t="n">
         <v>46314</v>
@@ -7548,7 +7548,7 @@
       </c>
       <c r="C124" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
         </is>
       </c>
       <c r="D124" s="78" t="inlineStr">
@@ -7557,7 +7557,7 @@
         </is>
       </c>
       <c r="E124" s="79" t="n">
-        <v>767367847.5204</v>
+        <v>4761468367.9458</v>
       </c>
       <c r="F124" s="77" t="n">
         <v>46314</v>
@@ -7582,7 +7582,7 @@
       </c>
       <c r="C125" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
         </is>
       </c>
       <c r="D125" s="78" t="inlineStr">
@@ -7591,7 +7591,7 @@
         </is>
       </c>
       <c r="E125" s="79" t="n">
-        <v>4761468367.9458</v>
+        <v>442076465.292</v>
       </c>
       <c r="F125" s="77" t="n">
         <v>46314</v>
@@ -7625,7 +7625,7 @@
         </is>
       </c>
       <c r="E126" s="79" t="n">
-        <v>442076465.292</v>
+        <v>444456984.744</v>
       </c>
       <c r="F126" s="77" t="n">
         <v>46314</v>
@@ -7641,7 +7641,7 @@
     </row>
     <row r="127">
       <c r="A127" s="77" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="B127" s="78" t="inlineStr">
         <is>
@@ -7650,7 +7650,7 @@
       </c>
       <c r="C127" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/45/2026</t>
         </is>
       </c>
       <c r="D127" s="78" t="inlineStr">
@@ -7659,13 +7659,13 @@
         </is>
       </c>
       <c r="E127" s="79" t="n">
-        <v>444456984.744</v>
+        <v>337392787.2479999</v>
       </c>
       <c r="F127" s="77" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="G127" s="80" t="n">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="H127" s="78" t="inlineStr">
         <is>
@@ -7684,7 +7684,7 @@
       </c>
       <c r="C128" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/45/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/46/2026</t>
         </is>
       </c>
       <c r="D128" s="78" t="inlineStr">
@@ -7693,7 +7693,7 @@
         </is>
       </c>
       <c r="E128" s="79" t="n">
-        <v>337392787.2479999</v>
+        <v>8211508178.4966</v>
       </c>
       <c r="F128" s="77" t="n">
         <v>46325</v>
@@ -7718,7 +7718,7 @@
       </c>
       <c r="C129" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/46/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/47/2026</t>
         </is>
       </c>
       <c r="D129" s="78" t="inlineStr">
@@ -7727,7 +7727,7 @@
         </is>
       </c>
       <c r="E129" s="79" t="n">
-        <v>8211508178.4966</v>
+        <v>903022062.8508</v>
       </c>
       <c r="F129" s="77" t="n">
         <v>46325</v>
@@ -7752,7 +7752,7 @@
       </c>
       <c r="C130" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/47/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/48/2026</t>
         </is>
       </c>
       <c r="D130" s="78" t="inlineStr">
@@ -7761,7 +7761,7 @@
         </is>
       </c>
       <c r="E130" s="79" t="n">
-        <v>903022062.8508</v>
+        <v>1912679476.3662</v>
       </c>
       <c r="F130" s="77" t="n">
         <v>46325</v>
@@ -7777,7 +7777,7 @@
     </row>
     <row r="131">
       <c r="A131" s="77" t="n">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="B131" s="78" t="inlineStr">
         <is>
@@ -7786,7 +7786,7 @@
       </c>
       <c r="C131" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/48/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/49/2026</t>
         </is>
       </c>
       <c r="D131" s="78" t="inlineStr">
@@ -7795,13 +7795,13 @@
         </is>
       </c>
       <c r="E131" s="79" t="n">
-        <v>1912679476.3662</v>
+        <v>479734948.6272</v>
       </c>
       <c r="F131" s="77" t="n">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="G131" s="80" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="H131" s="78" t="inlineStr">
         <is>
@@ -7820,7 +7820,7 @@
       </c>
       <c r="C132" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/49/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/50/2026</t>
         </is>
       </c>
       <c r="D132" s="78" t="inlineStr">
@@ -7829,7 +7829,7 @@
         </is>
       </c>
       <c r="E132" s="79" t="n">
-        <v>479734948.6272</v>
+        <v>3340238430.648</v>
       </c>
       <c r="F132" s="77" t="n">
         <v>46328</v>
@@ -7854,7 +7854,7 @@
       </c>
       <c r="C133" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/50/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/51/2026</t>
         </is>
       </c>
       <c r="D133" s="78" t="inlineStr">
@@ -7863,7 +7863,7 @@
         </is>
       </c>
       <c r="E133" s="79" t="n">
-        <v>3340238430.648</v>
+        <v>530510117.7436</v>
       </c>
       <c r="F133" s="77" t="n">
         <v>46328</v>
@@ -7879,7 +7879,7 @@
     </row>
     <row r="134">
       <c r="A134" s="77" t="n">
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="B134" s="78" t="inlineStr">
         <is>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="C134" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/51/2026</t>
+          <t>PT.PSI/PT.SSI/SWC/01/2026</t>
         </is>
       </c>
       <c r="D134" s="78" t="inlineStr">
@@ -7897,13 +7897,13 @@
         </is>
       </c>
       <c r="E134" s="79" t="n">
-        <v>530510117.7436</v>
+        <v>2345778403.95195</v>
       </c>
       <c r="F134" s="77" t="n">
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="G134" s="80" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="H134" s="78" t="inlineStr">
         <is>
@@ -7913,7 +7913,7 @@
     </row>
     <row r="135">
       <c r="A135" s="77" t="n">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="B135" s="78" t="inlineStr">
         <is>
@@ -7922,7 +7922,7 @@
       </c>
       <c r="C135" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/SWC/01/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
         </is>
       </c>
       <c r="D135" s="78" t="inlineStr">
@@ -7931,13 +7931,13 @@
         </is>
       </c>
       <c r="E135" s="79" t="n">
-        <v>2345778403.95195</v>
+        <v>3872356057.5561</v>
       </c>
       <c r="F135" s="77" t="n">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="G135" s="80" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H135" s="78" t="inlineStr">
         <is>
@@ -7965,7 +7965,7 @@
         </is>
       </c>
       <c r="E136" s="79" t="n">
-        <v>3872356057.5561</v>
+        <v>3951681440.2902</v>
       </c>
       <c r="F136" s="77" t="n">
         <v>46336</v>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="C137" s="78" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/53/IX/2026</t>
         </is>
       </c>
       <c r="D137" s="78" t="inlineStr">
@@ -7999,7 +7999,7 @@
         </is>
       </c>
       <c r="E137" s="79" t="n">
-        <v>3951681440.2902</v>
+        <v>539961649.7706</v>
       </c>
       <c r="F137" s="77" t="n">
         <v>46336</v>
@@ -8014,58 +8014,24 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="77" t="n">
-        <v>46336</v>
-      </c>
-      <c r="B138" s="78" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C138" s="78" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/53/IX/2026</t>
-        </is>
-      </c>
-      <c r="D138" s="78" t="inlineStr">
-        <is>
-          <t>Tolling</t>
-        </is>
-      </c>
-      <c r="E138" s="79" t="n">
-        <v>539961649.7706</v>
-      </c>
-      <c r="F138" s="77" t="n">
-        <v>46336</v>
-      </c>
-      <c r="G138" s="80" t="n">
-        <v>57</v>
-      </c>
-      <c r="H138" s="78" t="inlineStr">
-        <is>
-          <t>Future</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="40" t="inlineStr">
+      <c r="A138" s="40" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B139" s="81" t="n"/>
-      <c r="C139" s="81" t="n"/>
-      <c r="D139" s="81" t="n"/>
-      <c r="E139" s="82">
-        <f>SUM(E5:E138)</f>
+      <c r="B138" s="81" t="n"/>
+      <c r="C138" s="81" t="n"/>
+      <c r="D138" s="81" t="n"/>
+      <c r="E138" s="82">
+        <f>SUM(E5:E137)</f>
         <v/>
       </c>
-      <c r="F139" s="81" t="n"/>
-      <c r="G139" s="81" t="n"/>
-      <c r="H139" s="81" t="n"/>
+      <c r="F138" s="81" t="n"/>
+      <c r="G138" s="81" t="n"/>
+      <c r="H138" s="81" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H139"/>
+  <autoFilter ref="A4:H138"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13476,10 +13442,10 @@
         <v>-7295390.7099998</v>
       </c>
       <c r="BP30" s="87" t="n">
-        <v>1473357319.28</v>
+        <v>1705248424.64492</v>
       </c>
       <c r="BQ30" s="88" t="n">
-        <v>1583364434.94</v>
+        <v>1815255540.30492</v>
       </c>
       <c r="BR30" s="36" t="n">
         <v>-110007115.6600001</v>
@@ -13494,10 +13460,10 @@
         <v>1583364434.94</v>
       </c>
       <c r="BV30" s="41" t="n">
-        <v>25432859799.07084</v>
+        <v>25664750904.43576</v>
       </c>
       <c r="BW30" s="41" t="n">
-        <v>25422859799.07084</v>
+        <v>25654750904.43576</v>
       </c>
       <c r="BX30" s="41" t="n">
         <v>10000000</v>
@@ -15278,10 +15244,10 @@
         <v>-280418.0000000009</v>
       </c>
       <c r="BP39" s="91" t="n">
-        <v>4632523</v>
+        <v>4653413.8</v>
       </c>
       <c r="BQ39" s="92" t="n">
-        <v>5015461</v>
+        <v>5036351.8</v>
       </c>
       <c r="BR39" s="93" t="n">
         <v>-382938</v>
@@ -15296,10 +15262,10 @@
         <v>5015461</v>
       </c>
       <c r="BV39" s="94" t="n">
-        <v>45063181.53</v>
+        <v>45084072.33</v>
       </c>
       <c r="BW39" s="94" t="n">
-        <v>45063181.53</v>
+        <v>45084072.33</v>
       </c>
       <c r="BX39" s="94" t="n">
         <v>0</v>
@@ -16736,16 +16702,16 @@
         </is>
       </c>
       <c r="B16" s="36" t="n">
-        <v>50352917521.92064</v>
+        <v>50584808627.28556</v>
       </c>
       <c r="C16" s="36" t="n">
-        <v>46435325979.07042</v>
+        <v>46667217084.43534</v>
       </c>
       <c r="D16" s="99" t="n">
         <v>3917591542.85022</v>
       </c>
       <c r="E16" s="100" t="n">
-        <v>0.9221973276693504</v>
+        <v>0.9225539910269215</v>
       </c>
       <c r="F16" s="101" t="inlineStr">
         <is>
@@ -16856,7 +16822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1120"/>
+  <dimension ref="A1:Q1126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -78762,10 +78728,12 @@
       <c r="E979" s="106" t="n">
         <v>46278</v>
       </c>
-      <c r="F979" s="105" t="n"/>
+      <c r="F979" s="106" t="n">
+        <v>46279</v>
+      </c>
       <c r="G979" s="105" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H979" s="105" t="inlineStr">
@@ -78791,19 +78759,13 @@
       <c r="N979" s="107" t="n">
         <v>27842793.22</v>
       </c>
-      <c r="O979" s="105" t="n">
-        <v>1</v>
-      </c>
+      <c r="O979" s="105" t="n"/>
       <c r="P979" s="105" t="inlineStr">
         <is>
-          <t>OVERDUE 1</t>
-        </is>
-      </c>
-      <c r="Q979" s="105" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="Q979" s="105" t="n"/>
     </row>
     <row r="980">
       <c r="A980" s="105" t="inlineStr">
@@ -83606,7 +83568,7 @@
       </c>
       <c r="C1056" s="105" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/51/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/61/2026 </t>
         </is>
       </c>
       <c r="D1056" s="106" t="n">
@@ -83667,7 +83629,7 @@
       </c>
       <c r="C1057" s="105" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/52/2026 </t>
+          <t>PT.PSI/PT.ASI/FC/62/2026</t>
         </is>
       </c>
       <c r="D1057" s="106" t="n">
@@ -83728,7 +83690,7 @@
       </c>
       <c r="C1058" s="105" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/53/2026 </t>
+          <t>PT.PSI/PT.ASI/FC/63/2026</t>
         </is>
       </c>
       <c r="D1058" s="106" t="n">
@@ -85206,12 +85168,12 @@
       </c>
       <c r="B1081" s="105" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1081" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/13/2026</t>
+          <t>PT.PSI/PT.ASI/PIER-08/2026</t>
         </is>
       </c>
       <c r="D1081" s="106" t="n">
@@ -85220,15 +85182,17 @@
       <c r="E1081" s="106" t="n">
         <v>46295</v>
       </c>
-      <c r="F1081" s="105" t="n"/>
+      <c r="F1081" s="106" t="n">
+        <v>46265</v>
+      </c>
       <c r="G1081" s="105" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1081" s="105" t="inlineStr">
         <is>
-          <t>Rental CS</t>
+          <t>Rental - Chargeback</t>
         </is>
       </c>
       <c r="I1081" s="105" t="inlineStr">
@@ -85244,24 +85208,14 @@
         <v>46265</v>
       </c>
       <c r="M1081" s="107" t="n">
-        <v>5200</v>
+        <v>1</v>
       </c>
       <c r="N1081" s="107" t="n">
-        <v>872911811.2</v>
-      </c>
-      <c r="O1081" s="105" t="n">
-        <v>-16</v>
-      </c>
-      <c r="P1081" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1081" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
+        <v>10000000</v>
+      </c>
+      <c r="O1081" s="105" t="n"/>
+      <c r="P1081" s="105" t="n"/>
+      <c r="Q1081" s="105" t="n"/>
     </row>
     <row r="1082">
       <c r="A1082" s="105" t="inlineStr">
@@ -85271,12 +85225,12 @@
       </c>
       <c r="B1082" s="105" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1082" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/14/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-08/2026</t>
         </is>
       </c>
       <c r="D1082" s="106" t="n">
@@ -85285,15 +85239,17 @@
       <c r="E1082" s="106" t="n">
         <v>46295</v>
       </c>
-      <c r="F1082" s="105" t="n"/>
+      <c r="F1082" s="106" t="n">
+        <v>46265</v>
+      </c>
       <c r="G1082" s="105" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1082" s="105" t="inlineStr">
         <is>
-          <t>Rental CS</t>
+          <t>Rental WH, Office</t>
         </is>
       </c>
       <c r="I1082" s="105" t="inlineStr">
@@ -85309,24 +85265,14 @@
         <v>46265</v>
       </c>
       <c r="M1082" s="107" t="n">
-        <v>1800</v>
+        <v>1</v>
       </c>
       <c r="N1082" s="107" t="n">
-        <v>302161780.8</v>
-      </c>
-      <c r="O1082" s="105" t="n">
-        <v>-16</v>
-      </c>
-      <c r="P1082" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1082" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
+        <v>192258045</v>
+      </c>
+      <c r="O1082" s="105" t="n"/>
+      <c r="P1082" s="105" t="n"/>
+      <c r="Q1082" s="105" t="n"/>
     </row>
     <row r="1083">
       <c r="A1083" s="105" t="inlineStr">
@@ -85341,57 +85287,49 @@
       </c>
       <c r="C1083" s="105" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/66/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/RENTAL_MC-03/2026 </t>
         </is>
       </c>
       <c r="D1083" s="106" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="E1083" s="106" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F1083" s="105" t="n"/>
+        <v>46295</v>
+      </c>
+      <c r="F1083" s="106" t="n">
+        <v>46265</v>
+      </c>
       <c r="G1083" s="105" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1083" s="105" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Rental WH, Office</t>
         </is>
       </c>
       <c r="I1083" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1083" s="105" t="n"/>
       <c r="K1083" s="106" t="n">
-        <v>46206</v>
+        <v>46235</v>
       </c>
       <c r="L1083" s="106" t="n">
-        <v>46233</v>
+        <v>46265</v>
       </c>
       <c r="M1083" s="107" t="n">
-        <v>762117</v>
+        <v>1</v>
       </c>
       <c r="N1083" s="107" t="n">
-        <v>3100200501.96</v>
-      </c>
-      <c r="O1083" s="105" t="n">
-        <v>-17</v>
-      </c>
-      <c r="P1083" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1083" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
+        <v>6812450</v>
+      </c>
+      <c r="O1083" s="105" t="n"/>
+      <c r="P1083" s="105" t="n"/>
+      <c r="Q1083" s="105" t="n"/>
     </row>
     <row r="1084">
       <c r="A1084" s="105" t="inlineStr">
@@ -85406,57 +85344,49 @@
       </c>
       <c r="C1084" s="105" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
+          <t>PT.PSI/PT.ASI/PLN-08/2026</t>
         </is>
       </c>
       <c r="D1084" s="106" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="E1084" s="106" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F1084" s="105" t="n"/>
+        <v>46295</v>
+      </c>
+      <c r="F1084" s="106" t="n">
+        <v>46265</v>
+      </c>
       <c r="G1084" s="105" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1084" s="105" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Rental - Chargeback</t>
         </is>
       </c>
       <c r="I1084" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1084" s="105" t="n"/>
       <c r="K1084" s="106" t="n">
-        <v>46183</v>
+        <v>46235</v>
       </c>
       <c r="L1084" s="106" t="n">
-        <v>46183</v>
+        <v>46265</v>
       </c>
       <c r="M1084" s="107" t="n">
-        <v>150</v>
+        <v>16132.6</v>
       </c>
       <c r="N1084" s="107" t="n">
-        <v>237729</v>
-      </c>
-      <c r="O1084" s="105" t="n">
-        <v>-17</v>
-      </c>
-      <c r="P1084" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1084" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
+        <v>17211119.16084</v>
+      </c>
+      <c r="O1084" s="105" t="n"/>
+      <c r="P1084" s="105" t="n"/>
+      <c r="Q1084" s="105" t="n"/>
     </row>
     <row r="1085">
       <c r="A1085" s="105" t="inlineStr">
@@ -85471,57 +85401,49 @@
       </c>
       <c r="C1085" s="105" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
+          <t>PT.PSI/PT.ASI/PDAB-08/2026</t>
         </is>
       </c>
       <c r="D1085" s="106" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="E1085" s="106" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F1085" s="105" t="n"/>
+        <v>46295</v>
+      </c>
+      <c r="F1085" s="106" t="n">
+        <v>46265</v>
+      </c>
       <c r="G1085" s="105" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1085" s="105" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Rental - Chargeback</t>
         </is>
       </c>
       <c r="I1085" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1085" s="105" t="n"/>
       <c r="K1085" s="106" t="n">
-        <v>46230</v>
+        <v>46235</v>
       </c>
       <c r="L1085" s="106" t="n">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="M1085" s="107" t="n">
-        <v>89853</v>
+        <v>54</v>
       </c>
       <c r="N1085" s="107" t="n">
-        <v>142404425.58</v>
-      </c>
-      <c r="O1085" s="105" t="n">
-        <v>-17</v>
-      </c>
-      <c r="P1085" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1085" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
+        <v>594000</v>
+      </c>
+      <c r="O1085" s="105" t="n"/>
+      <c r="P1085" s="105" t="n"/>
+      <c r="Q1085" s="105" t="n"/>
     </row>
     <row r="1086">
       <c r="A1086" s="105" t="inlineStr">
@@ -85536,57 +85458,49 @@
       </c>
       <c r="C1086" s="105" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
+          <t>PT.PSI/PT.ASI_MC/PLN/02/2026</t>
         </is>
       </c>
       <c r="D1086" s="106" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="E1086" s="106" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F1086" s="105" t="n"/>
+        <v>46295</v>
+      </c>
+      <c r="F1086" s="106" t="n">
+        <v>46265</v>
+      </c>
       <c r="G1086" s="105" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1086" s="105" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Rental - Chargeback</t>
         </is>
       </c>
       <c r="I1086" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1086" s="105" t="n"/>
       <c r="K1086" s="106" t="n">
-        <v>46237</v>
+        <v>46235</v>
       </c>
       <c r="L1086" s="106" t="n">
-        <v>46242</v>
+        <v>46265</v>
       </c>
       <c r="M1086" s="107" t="n">
-        <v>170700</v>
+        <v>4701.2</v>
       </c>
       <c r="N1086" s="107" t="n">
-        <v>270535602</v>
-      </c>
-      <c r="O1086" s="105" t="n">
-        <v>-17</v>
-      </c>
-      <c r="P1086" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1086" s="105" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
+        <v>5015491.20408</v>
+      </c>
+      <c r="O1086" s="105" t="n"/>
+      <c r="P1086" s="105" t="n"/>
+      <c r="Q1086" s="105" t="n"/>
     </row>
     <row r="1087">
       <c r="A1087" s="105" t="inlineStr">
@@ -85596,19 +85510,19 @@
       </c>
       <c r="B1087" s="105" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1087" s="105" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/68/2026 </t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/13/2026</t>
         </is>
       </c>
       <c r="D1087" s="106" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="E1087" s="106" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="F1087" s="105" t="n"/>
       <c r="G1087" s="105" t="inlineStr">
@@ -85618,29 +85532,29 @@
       </c>
       <c r="H1087" s="105" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Rental CS</t>
         </is>
       </c>
       <c r="I1087" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1087" s="105" t="n"/>
       <c r="K1087" s="106" t="n">
-        <v>46218</v>
+        <v>46235</v>
       </c>
       <c r="L1087" s="106" t="n">
-        <v>46233</v>
+        <v>46265</v>
       </c>
       <c r="M1087" s="107" t="n">
-        <v>36342</v>
+        <v>5200</v>
       </c>
       <c r="N1087" s="107" t="n">
-        <v>28798491.06</v>
+        <v>872911811.2</v>
       </c>
       <c r="O1087" s="105" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="P1087" s="105" t="inlineStr">
         <is>
@@ -85666,14 +85580,14 @@
       </c>
       <c r="C1088" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/15/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/14/2026</t>
         </is>
       </c>
       <c r="D1088" s="106" t="n">
-        <v>46268</v>
+        <v>46265</v>
       </c>
       <c r="E1088" s="106" t="n">
-        <v>46298</v>
+        <v>46295</v>
       </c>
       <c r="F1088" s="105" t="n"/>
       <c r="G1088" s="105" t="inlineStr">
@@ -85693,19 +85607,19 @@
       </c>
       <c r="J1088" s="105" t="n"/>
       <c r="K1088" s="106" t="n">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="L1088" s="106" t="n">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="M1088" s="107" t="n">
-        <v>1657728.66</v>
+        <v>1800</v>
       </c>
       <c r="N1088" s="107" t="n">
-        <v>541504029.249372</v>
+        <v>302161780.8</v>
       </c>
       <c r="O1088" s="105" t="n">
-        <v>-19</v>
+        <v>-16</v>
       </c>
       <c r="P1088" s="105" t="inlineStr">
         <is>
@@ -85726,19 +85640,19 @@
       </c>
       <c r="B1089" s="105" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1089" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/49/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/66/2026 </t>
         </is>
       </c>
       <c r="D1089" s="106" t="n">
-        <v>46268</v>
+        <v>46266</v>
       </c>
       <c r="E1089" s="106" t="n">
-        <v>46328</v>
+        <v>46296</v>
       </c>
       <c r="F1089" s="105" t="n"/>
       <c r="G1089" s="105" t="inlineStr">
@@ -85758,19 +85672,19 @@
       </c>
       <c r="J1089" s="105" t="n"/>
       <c r="K1089" s="106" t="n">
-        <v>46258</v>
+        <v>46206</v>
       </c>
       <c r="L1089" s="106" t="n">
-        <v>46258</v>
+        <v>46233</v>
       </c>
       <c r="M1089" s="107" t="n">
-        <v>124152</v>
+        <v>762117</v>
       </c>
       <c r="N1089" s="107" t="n">
-        <v>479734948.6272</v>
+        <v>3100200501.96</v>
       </c>
       <c r="O1089" s="105" t="n">
-        <v>-49</v>
+        <v>-17</v>
       </c>
       <c r="P1089" s="105" t="inlineStr">
         <is>
@@ -85791,19 +85705,19 @@
       </c>
       <c r="B1090" s="105" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1090" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/50/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
         </is>
       </c>
       <c r="D1090" s="106" t="n">
-        <v>46268</v>
+        <v>46266</v>
       </c>
       <c r="E1090" s="106" t="n">
-        <v>46328</v>
+        <v>46296</v>
       </c>
       <c r="F1090" s="105" t="n"/>
       <c r="G1090" s="105" t="inlineStr">
@@ -85823,19 +85737,19 @@
       </c>
       <c r="J1090" s="105" t="n"/>
       <c r="K1090" s="106" t="n">
-        <v>46257</v>
+        <v>46183</v>
       </c>
       <c r="L1090" s="106" t="n">
-        <v>46261</v>
+        <v>46183</v>
       </c>
       <c r="M1090" s="107" t="n">
-        <v>864430</v>
+        <v>150</v>
       </c>
       <c r="N1090" s="107" t="n">
-        <v>3340238430.648</v>
+        <v>237729</v>
       </c>
       <c r="O1090" s="105" t="n">
-        <v>-49</v>
+        <v>-17</v>
       </c>
       <c r="P1090" s="105" t="inlineStr">
         <is>
@@ -85856,19 +85770,19 @@
       </c>
       <c r="B1091" s="105" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1091" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/51/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
         </is>
       </c>
       <c r="D1091" s="106" t="n">
-        <v>46268</v>
+        <v>46266</v>
       </c>
       <c r="E1091" s="106" t="n">
-        <v>46328</v>
+        <v>46296</v>
       </c>
       <c r="F1091" s="105" t="n"/>
       <c r="G1091" s="105" t="inlineStr">
@@ -85888,19 +85802,19 @@
       </c>
       <c r="J1091" s="105" t="n"/>
       <c r="K1091" s="106" t="n">
-        <v>46260</v>
+        <v>46230</v>
       </c>
       <c r="L1091" s="106" t="n">
-        <v>46262</v>
+        <v>46234</v>
       </c>
       <c r="M1091" s="107" t="n">
-        <v>38134</v>
+        <v>89853</v>
       </c>
       <c r="N1091" s="107" t="n">
-        <v>530510117.7436</v>
+        <v>142404425.58</v>
       </c>
       <c r="O1091" s="105" t="n">
-        <v>-49</v>
+        <v>-17</v>
       </c>
       <c r="P1091" s="105" t="inlineStr">
         <is>
@@ -85921,19 +85835,19 @@
       </c>
       <c r="B1092" s="105" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1092" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL OFFICE/03/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
         </is>
       </c>
       <c r="D1092" s="106" t="n">
-        <v>46268</v>
+        <v>46266</v>
       </c>
       <c r="E1092" s="106" t="n">
-        <v>46298</v>
+        <v>46296</v>
       </c>
       <c r="F1092" s="105" t="n"/>
       <c r="G1092" s="105" t="inlineStr">
@@ -85943,29 +85857,29 @@
       </c>
       <c r="H1092" s="105" t="inlineStr">
         <is>
-          <t>Rental Office</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1092" s="105" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1092" s="105" t="n"/>
       <c r="K1092" s="106" t="n">
-        <v>46174</v>
+        <v>46237</v>
       </c>
       <c r="L1092" s="106" t="n">
-        <v>46265</v>
+        <v>46242</v>
       </c>
       <c r="M1092" s="107" t="n">
-        <v>3</v>
+        <v>170700</v>
       </c>
       <c r="N1092" s="107" t="n">
-        <v>22509333.69</v>
+        <v>270535602</v>
       </c>
       <c r="O1092" s="105" t="n">
-        <v>-19</v>
+        <v>-17</v>
       </c>
       <c r="P1092" s="105" t="inlineStr">
         <is>
@@ -85986,19 +85900,19 @@
       </c>
       <c r="B1093" s="105" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1093" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/56/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/68/2026 </t>
         </is>
       </c>
       <c r="D1093" s="106" t="n">
-        <v>46274</v>
+        <v>46266</v>
       </c>
       <c r="E1093" s="106" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="F1093" s="105" t="n"/>
       <c r="G1093" s="105" t="inlineStr">
@@ -86018,19 +85932,19 @@
       </c>
       <c r="J1093" s="105" t="n"/>
       <c r="K1093" s="106" t="n">
-        <v>46204</v>
+        <v>46218</v>
       </c>
       <c r="L1093" s="106" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="M1093" s="107" t="n">
-        <v>19235.5</v>
+        <v>36342</v>
       </c>
       <c r="N1093" s="107" t="n">
-        <v>5535207.48</v>
+        <v>28798491.06</v>
       </c>
       <c r="O1093" s="105" t="n">
-        <v>-25</v>
+        <v>-17</v>
       </c>
       <c r="P1093" s="105" t="inlineStr">
         <is>
@@ -86056,14 +85970,14 @@
       </c>
       <c r="C1094" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/57/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/15/2026</t>
         </is>
       </c>
       <c r="D1094" s="106" t="n">
-        <v>46274</v>
+        <v>46268</v>
       </c>
       <c r="E1094" s="106" t="n">
-        <v>46304</v>
+        <v>46298</v>
       </c>
       <c r="F1094" s="105" t="n"/>
       <c r="G1094" s="105" t="inlineStr">
@@ -86073,29 +85987,29 @@
       </c>
       <c r="H1094" s="105" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Rental CS</t>
         </is>
       </c>
       <c r="I1094" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1094" s="105" t="n"/>
       <c r="K1094" s="106" t="n">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="L1094" s="106" t="n">
-        <v>46265</v>
+        <v>46234</v>
       </c>
       <c r="M1094" s="107" t="n">
-        <v>19753.5</v>
+        <v>1657728.66</v>
       </c>
       <c r="N1094" s="107" t="n">
-        <v>4392388.26</v>
+        <v>541504029.249372</v>
       </c>
       <c r="O1094" s="105" t="n">
-        <v>-25</v>
+        <v>-19</v>
       </c>
       <c r="P1094" s="105" t="inlineStr">
         <is>
@@ -86116,19 +86030,19 @@
       </c>
       <c r="B1095" s="105" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C1095" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/58/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/49/2026</t>
         </is>
       </c>
       <c r="D1095" s="106" t="n">
-        <v>46274</v>
+        <v>46268</v>
       </c>
       <c r="E1095" s="106" t="n">
-        <v>46304</v>
+        <v>46328</v>
       </c>
       <c r="F1095" s="105" t="n"/>
       <c r="G1095" s="105" t="inlineStr">
@@ -86148,19 +86062,19 @@
       </c>
       <c r="J1095" s="105" t="n"/>
       <c r="K1095" s="106" t="n">
-        <v>46204</v>
+        <v>46258</v>
       </c>
       <c r="L1095" s="106" t="n">
-        <v>46234</v>
+        <v>46258</v>
       </c>
       <c r="M1095" s="107" t="n">
-        <v>20874.3</v>
+        <v>124152</v>
       </c>
       <c r="N1095" s="107" t="n">
-        <v>18129124.98186</v>
+        <v>479734948.6272</v>
       </c>
       <c r="O1095" s="105" t="n">
-        <v>-25</v>
+        <v>-49</v>
       </c>
       <c r="P1095" s="105" t="inlineStr">
         <is>
@@ -86181,19 +86095,19 @@
       </c>
       <c r="B1096" s="105" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C1096" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/59/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/50/2026</t>
         </is>
       </c>
       <c r="D1096" s="106" t="n">
-        <v>46274</v>
+        <v>46268</v>
       </c>
       <c r="E1096" s="106" t="n">
-        <v>46304</v>
+        <v>46328</v>
       </c>
       <c r="F1096" s="105" t="n"/>
       <c r="G1096" s="105" t="inlineStr">
@@ -86213,19 +86127,19 @@
       </c>
       <c r="J1096" s="105" t="n"/>
       <c r="K1096" s="106" t="n">
-        <v>46235</v>
+        <v>46257</v>
       </c>
       <c r="L1096" s="106" t="n">
-        <v>46265</v>
+        <v>46261</v>
       </c>
       <c r="M1096" s="107" t="n">
-        <v>1625945.55</v>
+        <v>864430</v>
       </c>
       <c r="N1096" s="107" t="n">
-        <v>9884824431.36027</v>
+        <v>3340238430.648</v>
       </c>
       <c r="O1096" s="105" t="n">
-        <v>-25</v>
+        <v>-49</v>
       </c>
       <c r="P1096" s="105" t="inlineStr">
         <is>
@@ -86246,19 +86160,19 @@
       </c>
       <c r="B1097" s="105" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C1097" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/60/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/51/2026</t>
         </is>
       </c>
       <c r="D1097" s="106" t="n">
-        <v>46274</v>
+        <v>46268</v>
       </c>
       <c r="E1097" s="106" t="n">
-        <v>46304</v>
+        <v>46328</v>
       </c>
       <c r="F1097" s="105" t="n"/>
       <c r="G1097" s="105" t="inlineStr">
@@ -86278,19 +86192,19 @@
       </c>
       <c r="J1097" s="105" t="n"/>
       <c r="K1097" s="106" t="n">
-        <v>46235</v>
+        <v>46260</v>
       </c>
       <c r="L1097" s="106" t="n">
-        <v>46265</v>
+        <v>46262</v>
       </c>
       <c r="M1097" s="107" t="n">
-        <v>403173.25</v>
+        <v>38134</v>
       </c>
       <c r="N1097" s="107" t="n">
-        <v>700304033.0543</v>
+        <v>530510117.7436</v>
       </c>
       <c r="O1097" s="105" t="n">
-        <v>-25</v>
+        <v>-49</v>
       </c>
       <c r="P1097" s="105" t="inlineStr">
         <is>
@@ -86316,14 +86230,14 @@
       </c>
       <c r="C1098" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/61/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL OFFICE/03/2026</t>
         </is>
       </c>
       <c r="D1098" s="106" t="n">
-        <v>46274</v>
+        <v>46268</v>
       </c>
       <c r="E1098" s="106" t="n">
-        <v>46304</v>
+        <v>46298</v>
       </c>
       <c r="F1098" s="105" t="n"/>
       <c r="G1098" s="105" t="inlineStr">
@@ -86333,29 +86247,29 @@
       </c>
       <c r="H1098" s="105" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Rental Office</t>
         </is>
       </c>
       <c r="I1098" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1098" s="105" t="n"/>
       <c r="K1098" s="106" t="n">
-        <v>46235</v>
+        <v>46174</v>
       </c>
       <c r="L1098" s="106" t="n">
         <v>46265</v>
       </c>
       <c r="M1098" s="107" t="n">
-        <v>660572</v>
+        <v>3</v>
       </c>
       <c r="N1098" s="107" t="n">
-        <v>1147400616.7888</v>
+        <v>22509333.69</v>
       </c>
       <c r="O1098" s="105" t="n">
-        <v>-25</v>
+        <v>-19</v>
       </c>
       <c r="P1098" s="105" t="inlineStr">
         <is>
@@ -86381,7 +86295,7 @@
       </c>
       <c r="C1099" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/62/2026</t>
+          <t>PT.PSI/PT.CASI/REP/56/2026</t>
         </is>
       </c>
       <c r="D1099" s="106" t="n">
@@ -86408,16 +86322,16 @@
       </c>
       <c r="J1099" s="105" t="n"/>
       <c r="K1099" s="106" t="n">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="L1099" s="106" t="n">
-        <v>46265</v>
+        <v>46234</v>
       </c>
       <c r="M1099" s="107" t="n">
-        <v>5756</v>
+        <v>19235.5</v>
       </c>
       <c r="N1099" s="107" t="n">
-        <v>4999029.5912</v>
+        <v>5535207.48</v>
       </c>
       <c r="O1099" s="105" t="n">
         <v>-25</v>
@@ -86446,7 +86360,7 @@
       </c>
       <c r="C1100" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/63/2026</t>
+          <t>PT.PSI/PT.CASI/REP/57/2026</t>
         </is>
       </c>
       <c r="D1100" s="106" t="n">
@@ -86479,10 +86393,10 @@
         <v>46265</v>
       </c>
       <c r="M1100" s="107" t="n">
-        <v>40223</v>
+        <v>19753.5</v>
       </c>
       <c r="N1100" s="107" t="n">
-        <v>34933281.3146</v>
+        <v>4392388.26</v>
       </c>
       <c r="O1100" s="105" t="n">
         <v>-25</v>
@@ -86511,7 +86425,7 @@
       </c>
       <c r="C1101" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/64/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/58/2026</t>
         </is>
       </c>
       <c r="D1101" s="106" t="n">
@@ -86538,16 +86452,16 @@
       </c>
       <c r="J1101" s="105" t="n"/>
       <c r="K1101" s="106" t="n">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="L1101" s="106" t="n">
-        <v>46265</v>
+        <v>46234</v>
       </c>
       <c r="M1101" s="107" t="n">
-        <v>8166</v>
+        <v>20874.3</v>
       </c>
       <c r="N1101" s="107" t="n">
-        <v>85105002.66900001</v>
+        <v>18129124.98186</v>
       </c>
       <c r="O1101" s="105" t="n">
         <v>-25</v>
@@ -86576,7 +86490,7 @@
       </c>
       <c r="C1102" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/65/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/59/2026</t>
         </is>
       </c>
       <c r="D1102" s="106" t="n">
@@ -86609,10 +86523,10 @@
         <v>46265</v>
       </c>
       <c r="M1102" s="107" t="n">
-        <v>85023</v>
+        <v>1625945.55</v>
       </c>
       <c r="N1102" s="107" t="n">
-        <v>886098780.5445001</v>
+        <v>9884824431.36027</v>
       </c>
       <c r="O1102" s="105" t="n">
         <v>-25</v>
@@ -86641,7 +86555,7 @@
       </c>
       <c r="C1103" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/66/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/60/2026</t>
         </is>
       </c>
       <c r="D1103" s="106" t="n">
@@ -86674,10 +86588,10 @@
         <v>46265</v>
       </c>
       <c r="M1103" s="107" t="n">
-        <v>100.8</v>
+        <v>403173.25</v>
       </c>
       <c r="N1103" s="107" t="n">
-        <v>262631.43648</v>
+        <v>700304033.0543</v>
       </c>
       <c r="O1103" s="105" t="n">
         <v>-25</v>
@@ -86701,19 +86615,19 @@
       </c>
       <c r="B1104" s="105" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1104" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/SWC/01/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/61/2026</t>
         </is>
       </c>
       <c r="D1104" s="106" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="E1104" s="106" t="n">
-        <v>46335</v>
+        <v>46304</v>
       </c>
       <c r="F1104" s="105" t="n"/>
       <c r="G1104" s="105" t="inlineStr">
@@ -86733,19 +86647,19 @@
       </c>
       <c r="J1104" s="105" t="n"/>
       <c r="K1104" s="106" t="n">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="L1104" s="106" t="n">
-        <v>46173</v>
+        <v>46265</v>
       </c>
       <c r="M1104" s="107" t="n">
-        <v>46738.95</v>
+        <v>660572</v>
       </c>
       <c r="N1104" s="107" t="n">
-        <v>2345778403.95195</v>
+        <v>1147400616.7888</v>
       </c>
       <c r="O1104" s="105" t="n">
-        <v>-56</v>
+        <v>-25</v>
       </c>
       <c r="P1104" s="105" t="inlineStr">
         <is>
@@ -86766,19 +86680,19 @@
       </c>
       <c r="B1105" s="105" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1105" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-25/IX/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/62/2026</t>
         </is>
       </c>
       <c r="D1105" s="106" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="E1105" s="106" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="F1105" s="105" t="n"/>
       <c r="G1105" s="105" t="inlineStr">
@@ -86788,12 +86702,12 @@
       </c>
       <c r="H1105" s="105" t="inlineStr">
         <is>
-          <t>Rental CS -U2</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1105" s="105" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1105" s="105" t="n"/>
@@ -86804,13 +86718,13 @@
         <v>46265</v>
       </c>
       <c r="M1105" s="107" t="n">
-        <v>2309000</v>
+        <v>5756</v>
       </c>
       <c r="N1105" s="107" t="n">
-        <v>816231500</v>
+        <v>4999029.5912</v>
       </c>
       <c r="O1105" s="105" t="n">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="P1105" s="105" t="inlineStr">
         <is>
@@ -86831,19 +86745,19 @@
       </c>
       <c r="B1106" s="105" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1106" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/63/2026</t>
         </is>
       </c>
       <c r="D1106" s="106" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="E1106" s="106" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="F1106" s="105" t="n"/>
       <c r="G1106" s="105" t="inlineStr">
@@ -86853,12 +86767,12 @@
       </c>
       <c r="H1106" s="105" t="inlineStr">
         <is>
-          <t>Rental CS -U2</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1106" s="105" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1106" s="105" t="n"/>
@@ -86869,13 +86783,13 @@
         <v>46265</v>
       </c>
       <c r="M1106" s="107" t="n">
-        <v>506346</v>
+        <v>40223</v>
       </c>
       <c r="N1106" s="107" t="n">
-        <v>11590259.94</v>
+        <v>34933281.3146</v>
       </c>
       <c r="O1106" s="105" t="n">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="P1106" s="105" t="inlineStr">
         <is>
@@ -86896,19 +86810,19 @@
       </c>
       <c r="B1107" s="105" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1107" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/64/2026</t>
         </is>
       </c>
       <c r="D1107" s="106" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="E1107" s="106" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="F1107" s="105" t="n"/>
       <c r="G1107" s="105" t="inlineStr">
@@ -86918,12 +86832,12 @@
       </c>
       <c r="H1107" s="105" t="inlineStr">
         <is>
-          <t>Rental CS -U2</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1107" s="105" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1107" s="105" t="n"/>
@@ -86934,13 +86848,13 @@
         <v>46265</v>
       </c>
       <c r="M1107" s="107" t="n">
-        <v>115</v>
+        <v>8166</v>
       </c>
       <c r="N1107" s="107" t="n">
-        <v>62675</v>
+        <v>85105002.66900001</v>
       </c>
       <c r="O1107" s="105" t="n">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="P1107" s="105" t="inlineStr">
         <is>
@@ -86961,19 +86875,19 @@
       </c>
       <c r="B1108" s="105" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1108" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/27/IX/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/65/2026</t>
         </is>
       </c>
       <c r="D1108" s="106" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="E1108" s="106" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="F1108" s="105" t="n"/>
       <c r="G1108" s="105" t="inlineStr">
@@ -86983,12 +86897,12 @@
       </c>
       <c r="H1108" s="105" t="inlineStr">
         <is>
-          <t>Rental CS -U2</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1108" s="105" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1108" s="105" t="n"/>
@@ -86999,13 +86913,13 @@
         <v>46265</v>
       </c>
       <c r="M1108" s="107" t="n">
-        <v>2200000</v>
+        <v>85023</v>
       </c>
       <c r="N1108" s="107" t="n">
-        <v>755480000</v>
+        <v>886098780.5445001</v>
       </c>
       <c r="O1108" s="105" t="n">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="P1108" s="105" t="inlineStr">
         <is>
@@ -87026,19 +86940,19 @@
       </c>
       <c r="B1109" s="105" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1109" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/66/2026</t>
         </is>
       </c>
       <c r="D1109" s="106" t="n">
-        <v>46276</v>
+        <v>46274</v>
       </c>
       <c r="E1109" s="106" t="n">
-        <v>46336</v>
+        <v>46304</v>
       </c>
       <c r="F1109" s="105" t="n"/>
       <c r="G1109" s="105" t="inlineStr">
@@ -87058,19 +86972,19 @@
       </c>
       <c r="J1109" s="105" t="n"/>
       <c r="K1109" s="106" t="n">
-        <v>46261</v>
+        <v>46235</v>
       </c>
       <c r="L1109" s="106" t="n">
         <v>46265</v>
       </c>
       <c r="M1109" s="107" t="n">
-        <v>1011909</v>
+        <v>100.8</v>
       </c>
       <c r="N1109" s="107" t="n">
-        <v>3872356057.5561</v>
+        <v>262631.43648</v>
       </c>
       <c r="O1109" s="105" t="n">
-        <v>-57</v>
+        <v>-25</v>
       </c>
       <c r="P1109" s="105" t="inlineStr">
         <is>
@@ -87096,14 +87010,14 @@
       </c>
       <c r="C1110" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
+          <t>PT.PSI/PT.SSI/SWC/01/2026</t>
         </is>
       </c>
       <c r="D1110" s="106" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="E1110" s="106" t="n">
-        <v>46336</v>
+        <v>46335</v>
       </c>
       <c r="F1110" s="105" t="n"/>
       <c r="G1110" s="105" t="inlineStr">
@@ -87123,19 +87037,19 @@
       </c>
       <c r="J1110" s="105" t="n"/>
       <c r="K1110" s="106" t="n">
-        <v>46266</v>
+        <v>46143</v>
       </c>
       <c r="L1110" s="106" t="n">
-        <v>46271</v>
+        <v>46173</v>
       </c>
       <c r="M1110" s="107" t="n">
-        <v>1032638</v>
+        <v>46738.95</v>
       </c>
       <c r="N1110" s="107" t="n">
-        <v>3951681440.2902</v>
+        <v>2345778403.95195</v>
       </c>
       <c r="O1110" s="105" t="n">
-        <v>-57</v>
+        <v>-56</v>
       </c>
       <c r="P1110" s="105" t="inlineStr">
         <is>
@@ -87156,19 +87070,19 @@
       </c>
       <c r="B1111" s="105" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1111" s="105" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/53/IX/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-25/IX/2026</t>
         </is>
       </c>
       <c r="D1111" s="106" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="E1111" s="106" t="n">
-        <v>46336</v>
+        <v>46305</v>
       </c>
       <c r="F1111" s="105" t="n"/>
       <c r="G1111" s="105" t="inlineStr">
@@ -87178,29 +87092,29 @@
       </c>
       <c r="H1111" s="105" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Rental CS -U2</t>
         </is>
       </c>
       <c r="I1111" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1111" s="105" t="n"/>
       <c r="K1111" s="106" t="n">
-        <v>46267</v>
+        <v>46235</v>
       </c>
       <c r="L1111" s="106" t="n">
-        <v>46269</v>
+        <v>46265</v>
       </c>
       <c r="M1111" s="107" t="n">
-        <v>39198</v>
+        <v>2309000</v>
       </c>
       <c r="N1111" s="107" t="n">
-        <v>539961649.7706</v>
+        <v>816231500</v>
       </c>
       <c r="O1111" s="105" t="n">
-        <v>-57</v>
+        <v>-26</v>
       </c>
       <c r="P1111" s="105" t="inlineStr">
         <is>
@@ -87224,23 +87138,31 @@
           <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
-      <c r="C1112" s="105" t="n"/>
-      <c r="D1112" s="105" t="n"/>
-      <c r="E1112" s="105" t="n"/>
+      <c r="C1112" s="105" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1112" s="106" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E1112" s="106" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1112" s="105" t="n"/>
       <c r="G1112" s="105" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1112" s="105" t="inlineStr">
         <is>
-          <t>FC</t>
+          <t>Rental CS -U2</t>
         </is>
       </c>
       <c r="I1112" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1112" s="105" t="n"/>
@@ -87251,16 +87173,22 @@
         <v>46265</v>
       </c>
       <c r="M1112" s="107" t="n">
-        <v>3256990</v>
+        <v>506346</v>
       </c>
       <c r="N1112" s="107" t="n">
-        <v>13247943944.279</v>
-      </c>
-      <c r="O1112" s="105" t="n"/>
-      <c r="P1112" s="105" t="n"/>
+        <v>11590259.94</v>
+      </c>
+      <c r="O1112" s="105" t="n">
+        <v>-26</v>
+      </c>
+      <c r="P1112" s="105" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1112" s="105" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -87275,23 +87203,31 @@
           <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
-      <c r="C1113" s="105" t="n"/>
-      <c r="D1113" s="105" t="n"/>
-      <c r="E1113" s="105" t="n"/>
+      <c r="C1113" s="105" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1113" s="106" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E1113" s="106" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1113" s="105" t="n"/>
       <c r="G1113" s="105" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1113" s="105" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>Rental CS -U2</t>
         </is>
       </c>
       <c r="I1113" s="105" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1113" s="105" t="n"/>
@@ -87302,16 +87238,22 @@
         <v>46265</v>
       </c>
       <c r="M1113" s="107" t="n">
-        <v>140026</v>
+        <v>115</v>
       </c>
       <c r="N1113" s="107" t="n">
-        <v>1122459338.028</v>
-      </c>
-      <c r="O1113" s="105" t="n"/>
-      <c r="P1113" s="105" t="n"/>
+        <v>62675</v>
+      </c>
+      <c r="O1113" s="105" t="n">
+        <v>-26</v>
+      </c>
+      <c r="P1113" s="105" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1113" s="105" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -87323,21 +87265,29 @@
       </c>
       <c r="B1114" s="105" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1114" s="105" t="n"/>
-      <c r="D1114" s="105" t="n"/>
-      <c r="E1114" s="105" t="n"/>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1114" s="105" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/27/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1114" s="106" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E1114" s="106" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1114" s="105" t="n"/>
       <c r="G1114" s="105" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1114" s="105" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Rental CS -U2</t>
         </is>
       </c>
       <c r="I1114" s="105" t="inlineStr">
@@ -87353,16 +87303,22 @@
         <v>46265</v>
       </c>
       <c r="M1114" s="107" t="n">
-        <v>1654962.70767742</v>
+        <v>2200000</v>
       </c>
       <c r="N1114" s="107" t="n">
-        <v>593353779.5835853</v>
-      </c>
-      <c r="O1114" s="105" t="n"/>
-      <c r="P1114" s="105" t="n"/>
+        <v>755480000</v>
+      </c>
+      <c r="O1114" s="105" t="n">
+        <v>-26</v>
+      </c>
+      <c r="P1114" s="105" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1114" s="105" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -87377,43 +87333,57 @@
           <t>PT Syngenta Indonesia</t>
         </is>
       </c>
-      <c r="C1115" s="105" t="n"/>
-      <c r="D1115" s="105" t="n"/>
-      <c r="E1115" s="105" t="n"/>
+      <c r="C1115" s="105" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1115" s="106" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E1115" s="106" t="n">
+        <v>46336</v>
+      </c>
       <c r="F1115" s="105" t="n"/>
       <c r="G1115" s="105" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1115" s="105" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1115" s="105" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1115" s="105" t="n"/>
       <c r="K1115" s="106" t="n">
-        <v>46235</v>
+        <v>46261</v>
       </c>
       <c r="L1115" s="106" t="n">
         <v>46265</v>
       </c>
       <c r="M1115" s="107" t="n">
-        <v>1660000</v>
+        <v>1011909</v>
       </c>
       <c r="N1115" s="107" t="n">
-        <v>552691555.2</v>
-      </c>
-      <c r="O1115" s="105" t="n"/>
-      <c r="P1115" s="105" t="n"/>
+        <v>3872356057.5561</v>
+      </c>
+      <c r="O1115" s="105" t="n">
+        <v>-57</v>
+      </c>
+      <c r="P1115" s="105" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1115" s="105" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -87428,43 +87398,57 @@
           <t>PT Syngenta Indonesia</t>
         </is>
       </c>
-      <c r="C1116" s="105" t="n"/>
-      <c r="D1116" s="105" t="n"/>
-      <c r="E1116" s="105" t="n"/>
+      <c r="C1116" s="105" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1116" s="106" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E1116" s="106" t="n">
+        <v>46336</v>
+      </c>
       <c r="F1116" s="105" t="n"/>
       <c r="G1116" s="105" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1116" s="105" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1116" s="105" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1116" s="105" t="n"/>
       <c r="K1116" s="106" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="L1116" s="106" t="n">
-        <v>46265</v>
+        <v>46271</v>
       </c>
       <c r="M1116" s="107" t="n">
-        <v>1660000</v>
+        <v>1032638</v>
       </c>
       <c r="N1116" s="107" t="n">
-        <v>552691555.2</v>
-      </c>
-      <c r="O1116" s="105" t="n"/>
-      <c r="P1116" s="105" t="n"/>
+        <v>3951681440.2902</v>
+      </c>
+      <c r="O1116" s="105" t="n">
+        <v>-57</v>
+      </c>
+      <c r="P1116" s="105" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1116" s="105" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -87479,43 +87463,57 @@
           <t>PT Syngenta Indonesia</t>
         </is>
       </c>
-      <c r="C1117" s="105" t="n"/>
-      <c r="D1117" s="105" t="n"/>
-      <c r="E1117" s="105" t="n"/>
+      <c r="C1117" s="105" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/53/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1117" s="106" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E1117" s="106" t="n">
+        <v>46336</v>
+      </c>
       <c r="F1117" s="105" t="n"/>
       <c r="G1117" s="105" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1117" s="105" t="inlineStr">
         <is>
-          <t>RENTAL</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1117" s="105" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1117" s="105" t="n"/>
       <c r="K1117" s="106" t="n">
-        <v>46235</v>
+        <v>46267</v>
       </c>
       <c r="L1117" s="106" t="n">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="M1117" s="107" t="n">
-        <v>855000</v>
+        <v>39198</v>
       </c>
       <c r="N1117" s="107" t="n">
-        <v>71167361.40000001</v>
-      </c>
-      <c r="O1117" s="105" t="n"/>
-      <c r="P1117" s="105" t="n"/>
+        <v>539961649.7706</v>
+      </c>
+      <c r="O1117" s="105" t="n">
+        <v>-57</v>
+      </c>
+      <c r="P1117" s="105" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1117" s="105" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -87527,7 +87525,7 @@
       </c>
       <c r="B1118" s="105" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1118" s="105" t="n"/>
@@ -87541,12 +87539,12 @@
       </c>
       <c r="H1118" s="105" t="inlineStr">
         <is>
-          <t>RENTAL</t>
+          <t>FC</t>
         </is>
       </c>
       <c r="I1118" s="105" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1118" s="105" t="n"/>
@@ -87557,10 +87555,10 @@
         <v>46265</v>
       </c>
       <c r="M1118" s="107" t="n">
-        <v>3600000</v>
+        <v>3256990</v>
       </c>
       <c r="N1118" s="107" t="n">
-        <v>299652048</v>
+        <v>13247943944.279</v>
       </c>
       <c r="O1118" s="105" t="n"/>
       <c r="P1118" s="105" t="n"/>
@@ -87578,7 +87576,7 @@
       </c>
       <c r="B1119" s="105" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1119" s="105" t="n"/>
@@ -87592,7 +87590,7 @@
       </c>
       <c r="H1119" s="105" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="I1119" s="105" t="inlineStr">
@@ -87608,10 +87606,10 @@
         <v>46265</v>
       </c>
       <c r="M1119" s="107" t="n">
-        <v>855189</v>
+        <v>140026</v>
       </c>
       <c r="N1119" s="107" t="n">
-        <v>5789714193.710999</v>
+        <v>1122459338.028</v>
       </c>
       <c r="O1119" s="105" t="n"/>
       <c r="P1119" s="105" t="n"/>
@@ -87629,7 +87627,7 @@
       </c>
       <c r="B1120" s="105" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1120" s="105" t="n"/>
@@ -87659,10 +87657,10 @@
         <v>46265</v>
       </c>
       <c r="M1120" s="107" t="n">
-        <v>4000000</v>
+        <v>1654962.70767742</v>
       </c>
       <c r="N1120" s="107" t="n">
-        <v>1605326400</v>
+        <v>593353779.5835853</v>
       </c>
       <c r="O1120" s="105" t="n"/>
       <c r="P1120" s="105" t="n"/>
@@ -87672,8 +87670,314 @@
         </is>
       </c>
     </row>
+    <row r="1121">
+      <c r="A1121" s="105" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1121" s="105" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1121" s="105" t="n"/>
+      <c r="D1121" s="105" t="n"/>
+      <c r="E1121" s="105" t="n"/>
+      <c r="F1121" s="105" t="n"/>
+      <c r="G1121" s="105" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1121" s="105" t="inlineStr">
+        <is>
+          <t>RENTAL CS</t>
+        </is>
+      </c>
+      <c r="I1121" s="105" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1121" s="105" t="n"/>
+      <c r="K1121" s="106" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1121" s="106" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1121" s="107" t="n">
+        <v>1660000</v>
+      </c>
+      <c r="N1121" s="107" t="n">
+        <v>552691555.2</v>
+      </c>
+      <c r="O1121" s="105" t="n"/>
+      <c r="P1121" s="105" t="n"/>
+      <c r="Q1121" s="105" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="105" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1122" s="105" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1122" s="105" t="n"/>
+      <c r="D1122" s="105" t="n"/>
+      <c r="E1122" s="105" t="n"/>
+      <c r="F1122" s="105" t="n"/>
+      <c r="G1122" s="105" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1122" s="105" t="inlineStr">
+        <is>
+          <t>RENTAL CS</t>
+        </is>
+      </c>
+      <c r="I1122" s="105" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1122" s="105" t="n"/>
+      <c r="K1122" s="106" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1122" s="106" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1122" s="107" t="n">
+        <v>1660000</v>
+      </c>
+      <c r="N1122" s="107" t="n">
+        <v>552691555.2</v>
+      </c>
+      <c r="O1122" s="105" t="n"/>
+      <c r="P1122" s="105" t="n"/>
+      <c r="Q1122" s="105" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="105" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1123" s="105" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1123" s="105" t="n"/>
+      <c r="D1123" s="105" t="n"/>
+      <c r="E1123" s="105" t="n"/>
+      <c r="F1123" s="105" t="n"/>
+      <c r="G1123" s="105" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1123" s="105" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="I1123" s="105" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1123" s="105" t="n"/>
+      <c r="K1123" s="106" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1123" s="106" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1123" s="107" t="n">
+        <v>855000</v>
+      </c>
+      <c r="N1123" s="107" t="n">
+        <v>71167361.40000001</v>
+      </c>
+      <c r="O1123" s="105" t="n"/>
+      <c r="P1123" s="105" t="n"/>
+      <c r="Q1123" s="105" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="105" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1124" s="105" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1124" s="105" t="n"/>
+      <c r="D1124" s="105" t="n"/>
+      <c r="E1124" s="105" t="n"/>
+      <c r="F1124" s="105" t="n"/>
+      <c r="G1124" s="105" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1124" s="105" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="I1124" s="105" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1124" s="105" t="n"/>
+      <c r="K1124" s="106" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1124" s="106" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1124" s="107" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="N1124" s="107" t="n">
+        <v>299652048</v>
+      </c>
+      <c r="O1124" s="105" t="n"/>
+      <c r="P1124" s="105" t="n"/>
+      <c r="Q1124" s="105" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="105" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1125" s="105" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1125" s="105" t="n"/>
+      <c r="D1125" s="105" t="n"/>
+      <c r="E1125" s="105" t="n"/>
+      <c r="F1125" s="105" t="n"/>
+      <c r="G1125" s="105" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1125" s="105" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="I1125" s="105" t="inlineStr">
+        <is>
+          <t>Tolling</t>
+        </is>
+      </c>
+      <c r="J1125" s="105" t="n"/>
+      <c r="K1125" s="106" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1125" s="106" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1125" s="107" t="n">
+        <v>855189</v>
+      </c>
+      <c r="N1125" s="107" t="n">
+        <v>5789714193.710999</v>
+      </c>
+      <c r="O1125" s="105" t="n"/>
+      <c r="P1125" s="105" t="n"/>
+      <c r="Q1125" s="105" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="105" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1126" s="105" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1126" s="105" t="n"/>
+      <c r="D1126" s="105" t="n"/>
+      <c r="E1126" s="105" t="n"/>
+      <c r="F1126" s="105" t="n"/>
+      <c r="G1126" s="105" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1126" s="105" t="inlineStr">
+        <is>
+          <t>RENTAL CS</t>
+        </is>
+      </c>
+      <c r="I1126" s="105" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1126" s="105" t="n"/>
+      <c r="K1126" s="106" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1126" s="106" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1126" s="107" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="N1126" s="107" t="n">
+        <v>1605326400</v>
+      </c>
+      <c r="O1126" s="105" t="n"/>
+      <c r="P1126" s="105" t="n"/>
+      <c r="Q1126" s="105" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q1120"/>
+  <autoFilter ref="A1:Q1126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>